<commit_message>
Add key gen metrics
</commit_message>
<xml_diff>
--- a/results/all_optimizers_dnn_benchmarks.xlsx
+++ b/results/all_optimizers_dnn_benchmarks.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Original_RL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Without" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -458,11 +458,11 @@
     <col width="15" customWidth="1" min="11" max="11"/>
     <col width="13" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
     <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="25" customWidth="1" min="16" max="16"/>
-    <col width="110" customWidth="1" min="17" max="17"/>
-    <col width="149" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="112" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -571,35 +571,53 @@
       <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
-      <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
-      <c r="K2" s="2" t="inlineStr"/>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="n">
+        <v>7.9554</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>12.189</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>386.217</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>9.364000000000001</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>407.77</v>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>1.40075902787e-07</v>
+      </c>
       <c r="O2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>DSL generation exceeded the 10s timeout</t>
-        </is>
-      </c>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>C:\Users\Nazne\PFE\CHEHAB\Merged_Framework_2\CHEHAB\build\benchmarks\dnn_tensor\he\tensor_conv2d_auto.go</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -615,23 +633,45 @@
       <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="n">
+        <v>16.73</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>8.519</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>987.883</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>996.402</v>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>100900</v>
+      </c>
       <c r="O3" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>DSL_FAILED_3221226505</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -639,11 +679,7 @@
           <t>C:\Users\Nazne\PFE\CHEHAB\Merged_Framework_2\CHEHAB\build\benchmarks\dnn_tensor\he\tensor_full_dnn_auto.go</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>CRITICAL ERROR in optimizer (original_rl): std::bad_alloc terminate called after throwing an instance of 'std::bad_alloc' what():  std::bad_alloc</t>
-        </is>
-      </c>
+      <c r="R3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -659,35 +695,53 @@
       <c r="C4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr"/>
-      <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
-      <c r="L4" s="2" t="inlineStr"/>
-      <c r="M4" s="2" t="inlineStr"/>
-      <c r="N4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="n">
+        <v>14.0736</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>16.991</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>941.12</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>959.116</v>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="L4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N4" s="2" t="n">
+        <v>6669723.32603</v>
+      </c>
       <c r="O4" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr"/>
-      <c r="R4" s="2" t="inlineStr">
-        <is>
-          <t>DSL generation exceeded the 10s timeout</t>
-        </is>
-      </c>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>C:\Users\Nazne\PFE\CHEHAB\Merged_Framework_2\CHEHAB\build\benchmarks\dnn_tensor\he\tensor_cryptonets_auto.go</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -703,23 +757,45 @@
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
-      <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
-      <c r="L5" s="2" t="inlineStr"/>
-      <c r="M5" s="2" t="inlineStr"/>
-      <c r="N5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="n">
+        <v>534.683</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>6.959</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>2902.474</v>
+      </c>
+      <c r="G5" s="2" t="n">
+        <v>1.337</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>2910.77</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N5" s="2" t="n">
+        <v>20065.2718598</v>
+      </c>
       <c r="O5" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>DSL_FAILED_3221226505</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
@@ -727,11 +803,7 @@
           <t>C:\Users\Nazne\PFE\CHEHAB\Merged_Framework_2\CHEHAB\build\benchmarks\dnn_tensor\he\tensor_mlp_auto.go</t>
         </is>
       </c>
-      <c r="R5" s="2" t="inlineStr">
-        <is>
-          <t>CRITICAL ERROR in optimizer (original_rl): std::bad_alloc terminate called after throwing an instance of 'std::bad_alloc' what():  std::bad_alloc</t>
-        </is>
-      </c>
+      <c r="R5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -747,35 +819,53 @@
       <c r="C6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
-      <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
-      <c r="L6" s="2" t="inlineStr"/>
-      <c r="M6" s="2" t="inlineStr"/>
-      <c r="N6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="n">
+        <v>536.886</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>7.005</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>5619.562</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>1.014</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>5627.581</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>3019459.54439</v>
+      </c>
       <c r="O6" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>TIMEOUT</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr"/>
-      <c r="R6" s="2" t="inlineStr">
-        <is>
-          <t>DSL generation exceeded the 10s timeout</t>
-        </is>
-      </c>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>C:\Users\Nazne\PFE\CHEHAB\Merged_Framework_2\CHEHAB\build\benchmarks\dnn_tensor\he\tensor_lola_auto.go</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>